<commit_message>
Feature: Added smart column detection for excel reader
</commit_message>
<xml_diff>
--- a/test_data/sample_schedule.xlsx
+++ b/test_data/sample_schedule.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,10 +437,8 @@
           <t>Acme Corp</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
+      <c r="B2" s="1" t="n">
+        <v>46128</v>
       </c>
     </row>
     <row r="3">
@@ -446,10 +447,8 @@
           <t>Smith LLC</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
+      <c r="B3" s="1" t="n">
+        <v>46132</v>
       </c>
     </row>
     <row r="4">
@@ -458,10 +457,8 @@
           <t>Beta Inc</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
+      <c r="B4" s="1" t="n">
+        <v>46128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>